<commit_message>
Save accepted R3 publication masters, 13 product positions and owner approval
</commit_message>
<xml_diff>
--- a/products-storage/01-zakrytie-rabot/07-reestr-zamechaniy.xlsx
+++ b/products-storage/01-zakrytie-rabot/07-reestr-zamechaniy.xlsx
@@ -10,7 +10,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реестр" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Реестр'!$A$1:$K$103</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Реестр'!$1:$3</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -532,7 +535,7 @@
     <row r="2" ht="27" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Одна операция — одна строка. Заполните данные, затем отметьте результат и сохраните доказательства.</t>
+          <t xml:space="preserve">По каждому замечанию укажите содержание, документальное основание, позицию подрядчика, ответственного и срок. Устранение подтвердите актом, фотографией или иным документом.</t>
         </is>
       </c>
     </row>
@@ -1925,7 +1928,7 @@
     <row r="3" ht="108" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>1. Сделайте копию для объекта и назначьте владельца реестра. 2. Одна строка — одно замечание: укажите автора, работу/место, содержание и основание. 3. Запишите позицию подрядчика, ответственного и срок. 4. Обновляйте «Статус» вручную не реже двух раз в неделю. 5. При закрытии добавьте в «Доказательство закрытия» ссылку на акт, фото или иное подтверждение устранения. Не удаляйте историю замечания.</t>
+          <t xml:space="preserve">Зарегистрируйте каждое замечание с датой, автором, местом и основанием. Сопоставьте его с договором, проектом и актами. Укажите позицию подрядчика, ответственного и срок. При изменении статуса сохраните подтверждающий документ. История рассмотрения и устранения замечания сохраняется.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[skip deploy] Save owner-approved R3 production edition: eight systems and original P3 AOSR, 9 actual HTTP ZIPs / 123 verified buyer files
Scoped production release succeeded in run 39384126271. Approved buyer contents are immutable. Prices, 13-position catalog, emails and one-hour delivery verified. Preserve P5/P11/T2/T3 source trees. Four preexisting unrelated public-check failures remain explicitly classified in release evidence. General deployment intentionally skipped.
</commit_message>
<xml_diff>
--- a/products-storage/01-zakrytie-rabot/07-reestr-zamechaniy.xlsx
+++ b/products-storage/01-zakrytie-rabot/07-reestr-zamechaniy.xlsx
@@ -10,7 +10,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реестр" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Реестр'!$A$1:$K$103</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Реестр'!$1:$3</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -532,7 +535,7 @@
     <row r="2" ht="27" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Одна операция — одна строка. Заполните данные, затем отметьте результат и сохраните доказательства.</t>
+          <t xml:space="preserve">По каждому замечанию укажите содержание, документальное основание, позицию подрядчика, ответственного и срок. Устранение подтвердите актом, фотографией или иным документом.</t>
         </is>
       </c>
     </row>
@@ -1925,7 +1928,7 @@
     <row r="3" ht="108" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>1. Сделайте копию для объекта и назначьте владельца реестра. 2. Одна строка — одно замечание: укажите автора, работу/место, содержание и основание. 3. Запишите позицию подрядчика, ответственного и срок. 4. Обновляйте «Статус» вручную не реже двух раз в неделю. 5. При закрытии добавьте в «Доказательство закрытия» ссылку на акт, фото или иное подтверждение устранения. Не удаляйте историю замечания.</t>
+          <t xml:space="preserve">Зарегистрируйте каждое замечание с датой, автором, местом и основанием. Сопоставьте его с договором, проектом и актами. Укажите позицию подрядчика, ответственного и срок. При изменении статуса сохраните подтверждающий документ. История рассмотрения и устранения замечания сохраняется.</t>
         </is>
       </c>
     </row>

</xml_diff>